<commit_message>
feat: verify rule CG0082 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000024/negative/01/data/unit-test-coreid-CG0082-negative.xlsx
+++ b/rules/CORE-000024/negative/01/data/unit-test-coreid-CG0082-negative.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,6 +116,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -553,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -585,6 +594,159 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AEBDSYCD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Musculoskeletal and connective tissue disorders</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AEBDSYCD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Nervous system disorders</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AEBDSYCD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Vascular disorders</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1354,7 @@
           <t>Back pain</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Musculoskeletal and connective tissue disorders</t>
         </is>
@@ -1359,7 +1521,7 @@
           <t>Headache</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Nervous system disorders</t>
         </is>
@@ -1516,7 +1678,7 @@
           <t>Pulmonary embolism</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Vascular disorders</t>
         </is>

</xml_diff>